<commit_message>
sync: atualização automática 2026-06-02 16:40
</commit_message>
<xml_diff>
--- a/data/chamados.xlsx
+++ b/data/chamados.xlsx
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Verificacoes P1 e testes sistema som. Mic bancada OK. Mic sem fio com defeito plug carregamento. Cornetas necessitam troca bobinas. Bluetooth + Pre-Oneal funcionando perfeitamente.</t>
+          <t>Verificacoes P1 e testes sistema som. Mic bancada OK. Mic sem fio com defeito plug carregamento. Cornetas necessitam troca bobinas. Bluetooth + Pre-Oneal funcionando.</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>OS aberta. Atendimento nao realizado.</t>
+          <t>Orcamento emitido para substituicao do microfone sem fio Dylan UDX-02.</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1921,21 +1921,41 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
-        <is>
-          <t>Nao Atendido</t>
-        </is>
-      </c>
-      <c r="I18" s="16" t="inlineStr"/>
-      <c r="J18" s="17" t="inlineStr"/>
-      <c r="K18" s="17" t="inlineStr"/>
-      <c r="L18" s="16" t="inlineStr"/>
-      <c r="M18" s="16" t="inlineStr"/>
-      <c r="N18" s="16" t="inlineStr"/>
-      <c r="O18" s="16" t="inlineStr"/>
-      <c r="P18" s="17" t="inlineStr"/>
-      <c r="Q18" s="16" t="inlineStr"/>
-      <c r="R18" s="16" t="inlineStr"/>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Aguardando Aprovacao de Orcamento</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>25/05/2026</t>
+        </is>
+      </c>
+      <c r="J18" s="15" t="inlineStr">
+        <is>
+          <t>1x Mic Dylan UDX-02 Multi Dinamico Cardioide Preto S/Fio
+1x Servicos Tecnicos de Instalacao
+1x Mobilizacao de Equipe</t>
+        </is>
+      </c>
+      <c r="K18" s="15" t="inlineStr">
+        <is>
+          <t>R$1.107,86
+R$463,57
+R$282,86</t>
+        </is>
+      </c>
+      <c r="L18" s="14" t="inlineStr">
+        <is>
+          <t>R$ 1.854,29</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="inlineStr"/>
+      <c r="N18" s="14" t="inlineStr"/>
+      <c r="O18" s="14" t="inlineStr"/>
+      <c r="P18" s="15" t="inlineStr"/>
+      <c r="Q18" s="14" t="inlineStr"/>
+      <c r="R18" s="14" t="inlineStr"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
@@ -2183,7 +2203,8 @@
 Loja 42: R$ 1.335,71
 Loja 27: R$ 1.756,86
 Loja 12: R$ 1.282,14
-TOTAL: R$ 18.443,23</t>
+Loja 59: R$ 1.854,29
+TOTAL: R$ 20.297,52</t>
         </is>
       </c>
     </row>
@@ -2215,9 +2236,9 @@
     <row r="38"/>
     <row r="39"/>
     <row r="40"/>
+    <row r="41"/>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="I30:R40"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="I22:R28"/>
@@ -2226,6 +2247,7 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="A33:H33"/>
+    <mergeCell ref="I30:R41"/>
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A32:H32"/>

</xml_diff>